<commit_message>
fix: remove ununsed feature, add notif for product, pipelines
</commit_message>
<xml_diff>
--- a/public/documents/template_contacts.xlsx
+++ b/public/documents/template_contacts.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Template" sheetId="1" r:id="rId1"/>
+    <sheet name="Contacts" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:F2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -410,26 +410,38 @@
         <v>Phone</v>
       </c>
       <c r="D1" t="str">
+        <v>Company</v>
+      </c>
+      <c r="E1" t="str">
         <v>Position</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Address</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Contoh Nama</v>
+        <v>John Doe</v>
       </c>
       <c r="B2" t="str">
-        <v>email@contoh.com</v>
+        <v>john@example.com</v>
       </c>
       <c r="C2" t="str">
         <v>08123456789</v>
       </c>
       <c r="D2" t="str">
+        <v>Example Corp</v>
+      </c>
+      <c r="E2" t="str">
         <v>Manager</v>
+      </c>
+      <c r="F2" t="str">
+        <v>123 Main St, Jakarta</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>